<commit_message>
Reformat HH descriptions to match CMP convention
Format: '{Brand} {ProductName} - {Color} - {Size}'
Example: 'Helly Hansen Gilet Crew - Navy - S'

Previous version had a dash between brand and product name.
Now matches CMP format exactly: brand + space + product name,
then dash before color and size.

https://claude.ai/code/session_01CiHNiHv2TopSyFi729aDkF
</commit_message>
<xml_diff>
--- a/HellyHansen_EasyFatt_Import.xlsx
+++ b/HellyHansen_EasyFatt_Import.xlsx
@@ -696,7 +696,7 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>Helly Hansen - Gilet Crew - Navy - S</t>
+          <t>Helly Hansen Gilet Crew - Navy - S</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -769,7 +769,7 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>Helly Hansen - Gilet Crew - Navy - M</t>
+          <t>Helly Hansen Gilet Crew - Navy - M</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -842,7 +842,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Helly Hansen - Gilet Crew - Navy - L</t>
+          <t>Helly Hansen Gilet Crew - Navy - L</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -915,7 +915,7 @@
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Helly Hansen - Giacca Crew - Nero - S</t>
+          <t>Helly Hansen Giacca Crew - Nero - S</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -985,7 +985,7 @@
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>Helly Hansen - Giacca Crew - Nero - M</t>
+          <t>Helly Hansen Giacca Crew - Nero - M</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1055,7 +1055,7 @@
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Helly Hansen - Giacca Crew - Nero - L</t>
+          <t>Helly Hansen Giacca Crew - Nero - L</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1125,7 +1125,7 @@
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>Helly Hansen - Giacca Crew - Nero - XL</t>
+          <t>Helly Hansen Giacca Crew - Nero - XL</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2303,7 +2303,7 @@
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Grey Fog - 28</t>
+          <t>Helly Hansen Cargo Shorts - Grey Fog - 28</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2369,7 +2369,7 @@
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Grey Fog - 30</t>
+          <t>Helly Hansen Cargo Shorts - Grey Fog - 30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2435,7 +2435,7 @@
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Grey Fog - 32</t>
+          <t>Helly Hansen Cargo Shorts - Grey Fog - 32</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2501,7 +2501,7 @@
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Grey Fog - 33</t>
+          <t>Helly Hansen Cargo Shorts - Grey Fog - 33</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Grey Fog - 35</t>
+          <t>Helly Hansen Cargo Shorts - Grey Fog - 35</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2633,7 +2633,7 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Grey Fog - 36</t>
+          <t>Helly Hansen Cargo Shorts - Grey Fog - 36</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2699,7 +2699,7 @@
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Fallen Rock - 28</t>
+          <t>Helly Hansen Cargo Shorts - Fallen Rock - 28</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2769,7 +2769,7 @@
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Fallen Rock - 30</t>
+          <t>Helly Hansen Cargo Shorts - Fallen Rock - 30</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2839,7 +2839,7 @@
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Fallen Rock - 32</t>
+          <t>Helly Hansen Cargo Shorts - Fallen Rock - 32</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2905,7 +2905,7 @@
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>Helly Hansen - Cargo Shorts - Fallen Rock - 33</t>
+          <t>Helly Hansen Cargo Shorts - Fallen Rock - 33</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2971,7 +2971,7 @@
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>Helly Hansen - Club Shorts - Navy - 28</t>
+          <t>Helly Hansen Club Shorts - Navy - 28</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3037,7 +3037,7 @@
     <row r="36">
       <c r="B36" t="inlineStr">
         <is>
-          <t>Helly Hansen - Club Shorts - Navy - 32</t>
+          <t>Helly Hansen Club Shorts - Navy - 32</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3103,7 +3103,7 @@
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
-          <t>Helly Hansen - Club Shorts - Navy - 33</t>
+          <t>Helly Hansen Club Shorts - Navy - 33</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3169,7 +3169,7 @@
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>Helly Hansen - Club Shorts - Navy - 35</t>
+          <t>Helly Hansen Club Shorts - Navy - 35</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3235,7 +3235,7 @@
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>Helly Hansen - Club Shorts - Navy - 36</t>
+          <t>Helly Hansen Club Shorts - Navy - 36</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -3301,7 +3301,7 @@
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>Helly Hansen - Club Shorts - Navy - 38</t>
+          <t>Helly Hansen Club Shorts - Navy - 38</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">

</xml_diff>